<commit_message>
Correccion : Impedir reservas  para una fecha que tenga las mesas ocupadas y bloquear campos de entrada al asignar una mesa.
</commit_message>
<xml_diff>
--- a/HistorialReservasNew.xlsx
+++ b/HistorialReservasNew.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4635" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4635"/>
   </bookViews>
   <sheets>
     <sheet name="Historial" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <sheet name="Tablas" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlcn.WorksheetConnection_TablasA6B181" hidden="1">Tablas!$A$6:$B$18</definedName>
+    <definedName name="_xlcn.WorksheetConnection_TablasA6B18" hidden="1">Tablas!$A$6:$B$18</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -47,7 +47,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="Rango-00cd59a6-406c-4e0e-ae3e-646bcb50e1d8" autoDelete="1" usedByAddin="1">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_TablasA6B181"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_TablasA6B18"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="71">
   <si>
     <t>ID - Reserva</t>
   </si>
@@ -106,15 +106,6 @@
     <t>56478678</t>
   </si>
   <si>
-    <t>Carmita</t>
-  </si>
-  <si>
-    <t>48756456</t>
-  </si>
-  <si>
-    <t>15:00</t>
-  </si>
-  <si>
     <t>Jesus Martinez</t>
   </si>
   <si>
@@ -169,12 +160,6 @@
     <t>12:00</t>
   </si>
   <si>
-    <t>Daniel Gonzales</t>
-  </si>
-  <si>
-    <t>57896543</t>
-  </si>
-  <si>
     <t>16:00</t>
   </si>
   <si>
@@ -230,6 +215,60 @@
   </si>
   <si>
     <t xml:space="preserve">Mesas </t>
+  </si>
+  <si>
+    <t>Yoshio Arada Leon</t>
+  </si>
+  <si>
+    <t>56405717</t>
+  </si>
+  <si>
+    <t>Emilio Hernandez</t>
+  </si>
+  <si>
+    <t>54575891</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>Mario Paredes</t>
+  </si>
+  <si>
+    <t>56900971</t>
+  </si>
+  <si>
+    <t>Mario Portilla</t>
+  </si>
+  <si>
+    <t>56899090</t>
+  </si>
+  <si>
+    <t>Omar Menendez</t>
+  </si>
+  <si>
+    <t>52303898</t>
+  </si>
+  <si>
+    <t>Claudia Rodriguez</t>
+  </si>
+  <si>
+    <t>56784567</t>
+  </si>
+  <si>
+    <t>Lisandra Perez</t>
+  </si>
+  <si>
+    <t>54788090</t>
+  </si>
+  <si>
+    <t>Celina Galeano</t>
+  </si>
+  <si>
+    <t>54676776</t>
+  </si>
+  <si>
+    <t>03:00</t>
   </si>
 </sst>
 </file>
@@ -304,15 +343,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,13 +657,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>6</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -786,11 +823,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Reservaciones en</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Meses</a:t>
+              <a:t>Reservaciones en Meses</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -924,29 +957,6 @@
             <c:idx val="1"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:alpha val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                <a:solidFill>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="75000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-              <a:sp3d contourW="9525">
-                <a:contourClr>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="75000"/>
-                  </a:schemeClr>
-                </a:contourClr>
-              </a:sp3d>
-            </c:spPr>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -1002,13 +1012,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1048,12 +1058,12 @@
         </c:dLbls>
         <c:gapWidth val="65"/>
         <c:shape val="box"/>
-        <c:axId val="452316784"/>
-        <c:axId val="452317568"/>
+        <c:axId val="229692816"/>
+        <c:axId val="229693200"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="452316784"/>
+        <c:axId val="229692816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1088,7 +1098,7 @@
                     <a:lumOff val="25000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="Arial Rounded MT Bold" panose="020F0704030504030204" pitchFamily="34" charset="0"/>
+                <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -1096,7 +1106,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="452317568"/>
+        <c:crossAx val="229693200"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1104,7 +1114,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="452317568"/>
+        <c:axId val="229693200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1147,7 +1157,7 @@
                     <a:lumOff val="25000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="Arial Rounded MT Bold" panose="020F0704030504030204" pitchFamily="34" charset="0"/>
+                <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -1155,7 +1165,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="452316784"/>
+        <c:crossAx val="229692816"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1439,7 +1449,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1476,12 +1486,12 @@
         </c:dLbls>
         <c:gapWidth val="65"/>
         <c:shape val="box"/>
-        <c:axId val="455151128"/>
-        <c:axId val="455162888"/>
+        <c:axId val="229690768"/>
+        <c:axId val="229751776"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="455151128"/>
+        <c:axId val="229690768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1523,7 +1533,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="455162888"/>
+        <c:crossAx val="229751776"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1531,7 +1541,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="455162888"/>
+        <c:axId val="229751776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1579,7 +1589,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="455151128"/>
+        <c:crossAx val="229690768"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3964,7 +3974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -4007,25 +4017,25 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="4">
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="6">
         <v>46055</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>3</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>4</v>
       </c>
       <c r="H2" t="s">
@@ -4033,25 +4043,25 @@
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="A3">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="6">
         <v>46056</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>3</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>4</v>
       </c>
       <c r="H3" t="s">
@@ -4059,25 +4069,25 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="A4">
         <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="6">
         <v>46058</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>3</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>4</v>
       </c>
       <c r="H4" t="s">
@@ -4085,315 +4095,445 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>12</v>
+      <c r="A5">
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="4">
-        <v>46059</v>
-      </c>
-      <c r="E5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="1">
-        <v>6</v>
-      </c>
-      <c r="G5" s="1">
-        <v>5</v>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="6">
+        <v>46067</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="6">
+        <v>46067</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
         <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="4">
-        <v>46067</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="1">
-        <v>2</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>8</v>
+      <c r="A7">
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="4">
-        <v>46067</v>
-      </c>
-      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="6">
+        <v>46075</v>
+      </c>
+      <c r="E7" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="1">
-        <v>6</v>
-      </c>
-      <c r="G7" s="1">
-        <v>5</v>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>1</v>
+      <c r="A8">
+        <v>2</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="4">
-        <v>46075</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="D8" s="6">
+        <v>46081</v>
+      </c>
+      <c r="E8" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8">
         <v>3</v>
       </c>
-      <c r="G8" s="1">
-        <v>4</v>
+      <c r="G8">
+        <v>3</v>
       </c>
       <c r="H8" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>2</v>
+      <c r="A9">
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="4">
-        <v>46081</v>
-      </c>
-      <c r="E9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="6">
+        <v>46084</v>
+      </c>
+      <c r="E9" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="1">
-        <v>3</v>
-      </c>
-      <c r="G9" s="1">
-        <v>3</v>
+      <c r="F9">
+        <v>6</v>
+      </c>
+      <c r="G9">
+        <v>6</v>
       </c>
       <c r="H9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="A10">
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="4">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="6">
         <v>46085</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>8</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>11</v>
+      <c r="A11">
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="4">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="6">
         <v>46086</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="1">
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11">
         <v>3</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="A12">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
         <v>4</v>
       </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="4">
-        <v>46093</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="1">
-        <v>1</v>
-      </c>
-      <c r="G12" s="1">
-        <v>2</v>
-      </c>
       <c r="H12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>10</v>
+      <c r="A13">
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="4">
-        <v>46094</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="1">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13">
         <v>3</v>
       </c>
-      <c r="G13" s="1">
-        <v>3</v>
+      <c r="G13">
+        <v>4</v>
       </c>
       <c r="H13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>14</v>
+      <c r="A14">
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="4">
-        <v>46118</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F14" s="1">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14">
         <v>3</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14">
         <v>4</v>
       </c>
       <c r="H14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>9</v>
+      <c r="A15">
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="4">
-        <v>46125</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="1">
+        <v>64</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15">
         <v>3</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15">
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="A16">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="6">
+        <v>46086</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="6">
+        <v>46094</v>
+      </c>
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18">
+        <v>3</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="6">
+        <v>46095</v>
+      </c>
+      <c r="E19" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="6">
+        <v>46125</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="4">
+      <c r="B21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="6">
         <v>46179</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="1">
+      <c r="E21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21">
         <v>6</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G21">
         <v>5</v>
       </c>
-      <c r="H16" t="s">
-        <v>29</v>
+      <c r="H21" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -4426,22 +4566,22 @@
         <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>42</v>
+        <v>52</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1">
-        <f>COUNTIF(Historial!H:H,"Completada")</f>
-        <v>6</v>
+        <f>COUNTIF(Historial!H:H, "Pendiente")</f>
+        <v>11</v>
       </c>
       <c r="F2" s="1">
         <v>1</v>
@@ -4453,11 +4593,11 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1">
-        <f>COUNTIF(Historial!H:H,"Cancelada")</f>
-        <v>2</v>
+        <f>COUNTIF(Historial!H:H, "Cancelada")</f>
+        <v>4</v>
       </c>
       <c r="F3" s="1">
         <v>2</v>
@@ -4472,15 +4612,15 @@
         <v>10</v>
       </c>
       <c r="B4" s="1">
-        <f>COUNTIF(Historial!H:H,"Completada")</f>
-        <v>6</v>
+        <f>COUNTIF(Historial!H:H,  "Completada")</f>
+        <v>5</v>
       </c>
       <c r="F4" s="1">
         <v>3</v>
       </c>
       <c r="G4">
         <f>COUNTIF(Historial!F:F, "3")</f>
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4494,14 +4634,14 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="5">
+        <v>37</v>
+      </c>
+      <c r="D6" s="4">
         <f>MAX(B6:B17)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F6" s="1">
         <v>5</v>
@@ -4513,7 +4653,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B7" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,1,1),Historial!D:D, "&lt;="&amp;DATE(2026,1,31))</f>
@@ -4529,11 +4669,11 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,2,1),Historial!D:D, "&lt;="&amp;DATE(2026,2,29))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" s="1">
         <v>7</v>
@@ -4545,11 +4685,11 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B9" s="1">
-        <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,3,1),Historial!D:D, "&lt;="&amp;DATE(2026,3,31))</f>
-        <v>4</v>
+        <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,3,1), Historial!D:D, "&lt;="&amp;DATE(2026,3,31))</f>
+        <v>11</v>
       </c>
       <c r="F9" s="1">
         <v>8</v>
@@ -4561,11 +4701,11 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B10" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,4,1),Historial!D:D, "&lt;="&amp;DATE(2026,4,30))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="1">
         <v>9</v>
@@ -4577,7 +4717,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B11" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,5,1),Historial!D:D, "&lt;="&amp;DATE(2026,5,31))</f>
@@ -4593,7 +4733,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B12" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,6,1),Historial!D:D, "&lt;="&amp;DATE(2026,6,30))</f>
@@ -4602,7 +4742,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B13" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,7,1),Historial!D:D, "&lt;="&amp;DATE(2026,7,31))</f>
@@ -4611,7 +4751,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B14" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,8,1),Historial!D:D, "&lt;="&amp;DATE(2026,8,31))</f>
@@ -4620,7 +4760,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B15" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,9,1),Historial!D:D, "&lt;="&amp;DATE(2026,9,31))</f>
@@ -4629,7 +4769,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,10,1),Historial!D:D, "&lt;="&amp;DATE(2026,10,31))</f>
@@ -4638,7 +4778,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B17" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,11,1),Historial!D:D, "&lt;="&amp;DATE(2026,11,31))</f>
@@ -4647,7 +4787,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B18" s="1">
         <f>COUNTIFS(Historial!D:D, "&gt;="&amp;DATE(2026,12,1),Historial!D:D, "&lt;="&amp;DATE(2026,12,31))</f>
@@ -4656,7 +4796,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
-      <c r="B20" s="6"/>
+      <c r="B20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>